<commit_message>
New updates based on feedback
</commit_message>
<xml_diff>
--- a/files/unified_pipeline/unified_pipeline/data/results/cross_comparison.xlsx
+++ b/files/unified_pipeline/unified_pipeline/data/results/cross_comparison.xlsx
@@ -463,22 +463,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1414</v>
+        <v>0.1355</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1083</v>
+        <v>0.1028</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0167</v>
+        <v>0.0181</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1788</v>
+        <v>0.1821</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8298</v>
+        <v>0.824</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3449</v>
+        <v>0.3297</v>
       </c>
     </row>
     <row r="3">
@@ -488,22 +488,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7395</v>
+        <v>0.3738</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7358</v>
+        <v>0.3044</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6082</v>
+        <v>0.0808</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8398</v>
+        <v>0.3149</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9429</v>
+        <v>0.8627</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8497</v>
+        <v>0.6384</v>
       </c>
     </row>
     <row r="4">
@@ -513,22 +513,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2245</v>
+        <v>0.2072</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1973</v>
+        <v>0.1818</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0204</v>
+        <v>0.0152</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1935</v>
+        <v>0.192</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.8045</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4322</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="5">
@@ -538,22 +538,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4605</v>
+        <v>0.4761</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3694</v>
+        <v>0.3774</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0849</v>
+        <v>0.0936</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3909</v>
+        <v>0.4404</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8542</v>
+        <v>0.8615</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7012</v>
+        <v>0.7111</v>
       </c>
     </row>
     <row r="6">
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.09619999999999999</v>
+        <v>0.1125</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0824</v>
+        <v>0.09710000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0188</v>
+        <v>0.0242</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0776</v>
+        <v>0.1141</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8121</v>
+        <v>0.8087</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3042</v>
+        <v>0.3211</v>
       </c>
     </row>
   </sheetData>
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -639,22 +639,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3405</v>
+        <v>0.2796</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3073</v>
+        <v>0.2282</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1575</v>
+        <v>0.0487</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3446</v>
+        <v>0.2551</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8515</v>
+        <v>0.8384</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5391</v>
+        <v>0.5063</v>
       </c>
     </row>
     <row r="3">
@@ -664,22 +664,47 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3318</v>
+        <v>0.248</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3068</v>
+        <v>0.2035</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1866</v>
+        <v>0.0503</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3618</v>
+        <v>0.2385</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8551</v>
+        <v>0.8297</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4979</v>
+        <v>0.4481</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>qwen_coder</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.2407</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1953</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.2421</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.8252</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.4752</v>
       </c>
     </row>
   </sheetData>
@@ -740,22 +765,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3381</v>
+        <v>0.2592</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3072</v>
+        <v>0.2115</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1656</v>
+        <v>0.0458</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3494</v>
+        <v>0.2465</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8525</v>
+        <v>0.8321</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5276999999999999</v>
+        <v>0.4804</v>
       </c>
     </row>
   </sheetData>
@@ -769,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -826,22 +851,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1446</v>
+        <v>0.1428</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1114</v>
+        <v>0.1039</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0145</v>
+        <v>0.0156</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1865</v>
+        <v>0.1853</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8310999999999999</v>
+        <v>0.8312</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3687</v>
+        <v>0.3662</v>
       </c>
     </row>
     <row r="3">
@@ -851,138 +876,133 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1362</v>
+        <v>0.1252</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1033</v>
+        <v>0.0982</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0203</v>
+        <v>0.0199</v>
       </c>
       <c r="F3" t="n">
-        <v>0.166</v>
+        <v>0.179</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8277</v>
+        <v>0.8201000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3051</v>
+        <v>0.2747</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>qwen_coder</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1352</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1055</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1805</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.8176</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.331</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>codereval</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>groq</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>0.7582</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.7551</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.6462</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.8477</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.9494</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.8826000000000001</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="n">
+        <v>0.4139</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.3423</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0931</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.3207</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.8749</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.6818</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
         <is>
           <t>huggingface</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>0.7082000000000001</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.7035</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.5448</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.8266</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9322</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.7948</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>funcom</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>groq</t>
-        </is>
-      </c>
       <c r="C6" t="n">
-        <v>0.2311</v>
+        <v>0.3498</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2069</v>
+        <v>0.2876</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0232</v>
+        <v>0.0759</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2027</v>
+        <v>0.2883</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8086</v>
+        <v>0.8612</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4247</v>
+        <v>0.5747</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>huggingface</t>
+          <t>qwen_coder</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.2012</v>
+        <v>0.3461</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1631</v>
+        <v>0.2723</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0105</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1607</v>
+        <v>0.3352</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8057</v>
+        <v>0.8481</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4591</v>
+        <v>0.6483</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>robustness_copilot</t>
+          <t>funcom</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -991,22 +1011,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.4782</v>
+        <v>0.23</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3892</v>
+        <v>0.1977</v>
       </c>
       <c r="E8" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0203</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4104</v>
+        <v>0.2174</v>
       </c>
       <c r="G8" t="n">
-        <v>0.8581</v>
+        <v>0.8106</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7197</v>
+        <v>0.4279</v>
       </c>
     </row>
     <row r="9">
@@ -1016,86 +1036,216 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.3132</v>
+        <v>0.1889</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2049</v>
+        <v>0.1641</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0517</v>
+        <v>0.0108</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2279</v>
+        <v>0.1818</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8215</v>
+        <v>0.8001</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5469000000000001</v>
+        <v>0.3911</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>qwen_coder</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1953</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.1787</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.0128</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1689</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.801</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.4053</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>robustness_copilot</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.4816</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.3869</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0825</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.8605</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.7155</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>huggingface</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.5004999999999999</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.3944</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1348</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.4768</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.8617</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.695</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>qwen_coder</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4441</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.3455</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0736</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.863</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.7186</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>tesoro</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>groq</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>0.0906</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.0741</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.0148</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.0756</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.8103</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.2997</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="C14" t="n">
+        <v>0.1298</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.0319</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.1261</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.8151</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.3401</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
         <is>
           <t>huggingface</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>0.1138</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.1082</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.0311</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.0839</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.8176</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.3184</v>
+      <c r="C15" t="n">
+        <v>0.1006</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.0902</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.0235</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.0983</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.8077</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3257</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>qwen_coder</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.0974</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.0838</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.1112</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.7999000000000001</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.2867</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A14:A16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>